<commit_message>
Migliora ARIMA: forecast 252 passi, rendimenti log, correzione Jensen; fix drawdown callback; aggiorna TARBIUTH
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portafoglio/TARBIUTH.xlsx
+++ b/portafoglio/TARBIUTH.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbookpro/Downloads/andcappe_zip/Dashboard/SITO_WEB/Sito personale/portafoglio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD18DA53-BB77-FD44-8EF3-25BCC7170B0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BC11CF7-0E93-5940-A76B-7711893FA9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4380" yWindow="20" windowWidth="24420" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4380" yWindow="0" windowWidth="24420" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio21" sheetId="29" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7586" uniqueCount="2753">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7586" uniqueCount="2756">
   <si>
     <t>Simbolo</t>
   </si>
@@ -8554,9 +8554,6 @@
     <t xml:space="preserve">Gold </t>
   </si>
   <si>
-    <t>AZ. VANGUARD ACWI</t>
-  </si>
-  <si>
     <t>Azionario ACWI Vanguard</t>
   </si>
   <si>
@@ -8569,7 +8566,19 @@
     <t>JEGA.MI</t>
   </si>
   <si>
-    <t>Premium Income Active</t>
+    <t>Alt. MF</t>
+  </si>
+  <si>
+    <t>Alt. Inf.Br.</t>
+  </si>
+  <si>
+    <t>Alt. Eu.Def</t>
+  </si>
+  <si>
+    <t>Alt. Pr.Inc.Ac</t>
+  </si>
+  <si>
+    <t>Bench AZ. VANGUARD ACWI</t>
   </si>
 </sst>
 </file>
@@ -9253,28 +9262,24 @@
       <name val="Abadi"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Abadi"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF232A31"/>
       <name val="Abadi"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="8"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Abadi"/>
     </font>
     <font>
-      <b/>
       <u/>
-      <sz val="9"/>
+      <sz val="11"/>
       <color theme="10"/>
-      <name val="Abadi"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
       <name val="Abadi"/>
     </font>
   </fonts>
@@ -9877,6 +9882,13 @@
     <xf numFmtId="0" fontId="98" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="101" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="101" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="101" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="85" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -9887,29 +9899,22 @@
     <xf numFmtId="0" fontId="83" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="101" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="102" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="101" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="101" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="102" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="103" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="102" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="103" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="102" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="103" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="104" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="105" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="104" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="103" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="105" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="102" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="104" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="105" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -9920,7 +9925,7 @@
   <dxfs count="12">
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -9929,7 +9934,7 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="9"/>
+        <sz val="11"/>
         <color indexed="8"/>
         <name val="Abadi"/>
         <scheme val="none"/>
@@ -9937,7 +9942,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -9946,7 +9951,7 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="9"/>
+        <sz val="11"/>
         <color indexed="8"/>
         <name val="Abadi"/>
         <scheme val="none"/>
@@ -9954,7 +9959,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -9963,7 +9968,7 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="9"/>
+        <sz val="11"/>
         <color indexed="8"/>
         <name val="Abadi"/>
         <scheme val="none"/>
@@ -9971,7 +9976,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -9980,7 +9985,7 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="9"/>
+        <sz val="11"/>
         <color indexed="8"/>
         <name val="Abadi"/>
         <scheme val="none"/>
@@ -9988,7 +9993,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -9997,19 +10002,8 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="9"/>
+        <sz val="11"/>
         <color indexed="8"/>
-        <name val="Abadi"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
         <name val="Abadi"/>
         <scheme val="none"/>
       </font>
@@ -10114,6 +10108,17 @@
         <name val="Helvetica Neue"/>
         <family val="2"/>
         <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <name val="Abadi"/>
+        <scheme val="none"/>
       </font>
     </dxf>
   </dxfs>
@@ -16299,7 +16304,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}" name="Tabella32" displayName="Tabella32" ref="A1:D30" totalsRowShown="0" headerRowDxfId="5" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}" name="Tabella32" displayName="Tabella32" ref="A1:D30" totalsRowShown="0" headerRowDxfId="11" dataDxfId="0">
   <autoFilter ref="A1:D30" xr:uid="{246183AC-3204-9D4E-95E8-61DE399D8F79}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{12AF85F4-CF3E-1A44-9197-52CD700ECF69}" name="SIMBOLO" dataDxfId="4"/>
@@ -16312,13 +16317,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{48919E7F-61A8-DB47-85A6-D1B66A3AD480}" name="Tabella323" displayName="Tabella323" ref="A1:D53" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{48919E7F-61A8-DB47-85A6-D1B66A3AD480}" name="Tabella323" displayName="Tabella323" ref="A1:D53" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:D53" xr:uid="{48919E7F-61A8-DB47-85A6-D1B66A3AD480}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{99BE53A6-82BE-7C4C-8EDB-FC2585DE7E29}" name="SIMBOLO" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{79CB9D70-57D7-004E-8DD2-11CA0A269F24}" name="DESCRIZIONE" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{4221CAB4-B4C0-5746-BDF4-C3FC111D5F78}" name="VALUTA" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{530400BE-E6AA-4A47-B046-BF29D0205198}" name="CLASSE" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{99BE53A6-82BE-7C4C-8EDB-FC2585DE7E29}" name="SIMBOLO" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{79CB9D70-57D7-004E-8DD2-11CA0A269F24}" name="DESCRIZIONE" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{4221CAB4-B4C0-5746-BDF4-C3FC111D5F78}" name="VALUTA" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{530400BE-E6AA-4A47-B046-BF29D0205198}" name="CLASSE" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -17432,428 +17437,428 @@
   <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="11"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" style="237" customWidth="1"/>
-    <col min="2" max="2" width="106.5" style="237" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="237"/>
+    <col min="1" max="1" width="11.83203125" style="233" customWidth="1"/>
+    <col min="2" max="2" width="106.5" style="233" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="233"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="235" t="s">
+      <c r="A1" s="231" t="s">
         <v>2120</v>
       </c>
-      <c r="B1" s="236" t="s">
+      <c r="B1" s="232" t="s">
         <v>2121</v>
       </c>
-      <c r="C1" s="237" t="s">
+      <c r="C1" s="233" t="s">
         <v>2122</v>
       </c>
-      <c r="D1" s="237" t="s">
+      <c r="D1" s="233" t="s">
         <v>2703</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="239" t="s">
+    <row r="2" spans="1:4" ht="12">
+      <c r="A2" s="238" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="240" t="s">
+      <c r="B2" s="239" t="s">
+        <v>2755</v>
+      </c>
+      <c r="C2" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="240" t="s">
         <v>2747</v>
       </c>
-      <c r="C2" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="241" t="s">
+    </row>
+    <row r="3" spans="1:4" ht="12">
+      <c r="A3" s="241" t="s">
+        <v>2571</v>
+      </c>
+      <c r="B3" s="241" t="s">
+        <v>2751</v>
+      </c>
+      <c r="C3" s="242" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="243" t="s">
+        <v>2723</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="12">
+      <c r="A4" s="240" t="s">
+        <v>2255</v>
+      </c>
+      <c r="B4" s="241" t="s">
+        <v>2753</v>
+      </c>
+      <c r="C4" s="244" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="243" t="s">
+        <v>2723</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="12">
+      <c r="A5" s="241" t="s">
+        <v>2750</v>
+      </c>
+      <c r="B5" s="241" t="s">
+        <v>2754</v>
+      </c>
+      <c r="C5" s="244" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="243" t="s">
+        <v>2723</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="12">
+      <c r="A6" s="240" t="s">
+        <v>2617</v>
+      </c>
+      <c r="B6" s="241" t="s">
+        <v>2752</v>
+      </c>
+      <c r="C6" s="244" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="243" t="s">
+        <v>2723</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="12">
+      <c r="A7" s="238" t="s">
+        <v>2619</v>
+      </c>
+      <c r="B7" s="241" t="s">
+        <v>2724</v>
+      </c>
+      <c r="C7" s="240" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="240" t="s">
+        <v>2696</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="12">
+      <c r="A8" s="240" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B8" s="241" t="s">
+        <v>2734</v>
+      </c>
+      <c r="C8" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="240" t="s">
+        <v>2635</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="12">
+      <c r="A9" s="240" t="s">
+        <v>2706</v>
+      </c>
+      <c r="B9" s="241" t="s">
+        <v>2731</v>
+      </c>
+      <c r="C9" s="240" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="240" t="s">
+        <v>2708</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="12">
+      <c r="A10" s="240" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="240" t="s">
         <v>2748</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="238" t="s">
-        <v>2571</v>
-      </c>
-      <c r="B3" s="238" t="s">
-        <v>2572</v>
-      </c>
-      <c r="C3" s="243" t="s">
-        <v>28</v>
-      </c>
-      <c r="D3" s="244" t="s">
-        <v>2723</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="241" t="s">
-        <v>2255</v>
-      </c>
-      <c r="B4" s="238" t="s">
-        <v>2614</v>
-      </c>
-      <c r="C4" s="245" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="244" t="s">
-        <v>2723</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="45">
-      <c r="A5" s="180" t="s">
-        <v>2751</v>
-      </c>
-      <c r="B5" s="180" t="s">
-        <v>2752</v>
-      </c>
-      <c r="C5" s="245" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="244" t="s">
-        <v>2723</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="241" t="s">
-        <v>2617</v>
-      </c>
-      <c r="B6" s="238" t="s">
-        <v>2618</v>
-      </c>
-      <c r="C6" s="245" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="244" t="s">
-        <v>2723</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="239" t="s">
-        <v>2619</v>
-      </c>
-      <c r="B7" s="238" t="s">
-        <v>2724</v>
-      </c>
-      <c r="C7" s="241" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" s="241" t="s">
-        <v>2696</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="241" t="s">
-        <v>1091</v>
-      </c>
-      <c r="B8" s="238" t="s">
-        <v>2734</v>
-      </c>
-      <c r="C8" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="241" t="s">
-        <v>2635</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="241" t="s">
-        <v>2706</v>
-      </c>
-      <c r="B9" s="238" t="s">
-        <v>2731</v>
-      </c>
-      <c r="C9" s="241" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="241" t="s">
-        <v>2708</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="241" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" s="241" t="s">
+      <c r="C10" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="240" t="s">
         <v>2749</v>
       </c>
-      <c r="C10" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="241" t="s">
-        <v>2750</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="241" t="s">
+    </row>
+    <row r="11" spans="1:4" ht="12">
+      <c r="A11" s="240" t="s">
         <v>2668</v>
       </c>
-      <c r="B11" s="241" t="s">
+      <c r="B11" s="240" t="s">
         <v>2725</v>
       </c>
-      <c r="C11" s="241" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="241" t="s">
+      <c r="C11" s="240" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="240" t="s">
         <v>2673</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="241" t="s">
+    <row r="12" spans="1:4" ht="12">
+      <c r="A12" s="240" t="s">
         <v>1089</v>
       </c>
-      <c r="B12" s="241" t="s">
+      <c r="B12" s="240" t="s">
         <v>2726</v>
       </c>
-      <c r="C12" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="241" t="s">
+      <c r="C12" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="240" t="s">
         <v>2680</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="242" t="s">
+    <row r="13" spans="1:4" ht="12">
+      <c r="A13" s="245" t="s">
         <v>2704</v>
       </c>
-      <c r="B13" s="241" t="s">
+      <c r="B13" s="240" t="s">
         <v>2727</v>
       </c>
-      <c r="C13" s="241" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="241" t="s">
+      <c r="C13" s="240" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="240" t="s">
         <v>2685</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="241" t="s">
+    <row r="14" spans="1:4" ht="12">
+      <c r="A14" s="240" t="s">
         <v>2681</v>
       </c>
-      <c r="B14" s="241" t="s">
+      <c r="B14" s="240" t="s">
         <v>2728</v>
       </c>
-      <c r="C14" s="241" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="241" t="s">
+      <c r="C14" s="240" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="240" t="s">
         <v>2686</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="241" t="s">
+    <row r="15" spans="1:4" ht="12">
+      <c r="A15" s="240" t="s">
         <v>2683</v>
       </c>
-      <c r="B15" s="241" t="s">
+      <c r="B15" s="240" t="s">
         <v>2729</v>
       </c>
-      <c r="C15" s="241" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="241" t="s">
+      <c r="C15" s="240" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="240" t="s">
         <v>2687</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="242" t="s">
+    <row r="16" spans="1:4" ht="12">
+      <c r="A16" s="245" t="s">
         <v>20</v>
       </c>
-      <c r="B16" s="241" t="s">
+      <c r="B16" s="240" t="s">
         <v>2730</v>
       </c>
-      <c r="C16" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D16" s="241" t="s">
+      <c r="C16" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="240" t="s">
         <v>2691</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="241" t="s">
+    <row r="17" spans="1:4" ht="12">
+      <c r="A17" s="240" t="s">
         <v>1872</v>
       </c>
-      <c r="B17" s="241" t="s">
+      <c r="B17" s="240" t="s">
         <v>2733</v>
       </c>
-      <c r="C17" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="241" t="s">
+      <c r="C17" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="240" t="s">
         <v>2694</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="241" t="s">
+    <row r="18" spans="1:4" ht="12">
+      <c r="A18" s="240" t="s">
         <v>833</v>
       </c>
-      <c r="B18" s="241" t="s">
+      <c r="B18" s="240" t="s">
         <v>2732</v>
       </c>
-      <c r="C18" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="241" t="s">
+      <c r="C18" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="240" t="s">
         <v>2692</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="241" t="s">
+    <row r="19" spans="1:4" ht="12">
+      <c r="A19" s="240" t="s">
         <v>2636</v>
       </c>
-      <c r="B19" s="241" t="s">
+      <c r="B19" s="240" t="s">
         <v>2735</v>
       </c>
-      <c r="C19" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D19" s="241" t="s">
+      <c r="C19" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="240" t="s">
         <v>2640</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="241" t="s">
+    <row r="20" spans="1:4" ht="12">
+      <c r="A20" s="240" t="s">
         <v>1090</v>
       </c>
-      <c r="B20" s="241" t="s">
+      <c r="B20" s="240" t="s">
         <v>2736</v>
       </c>
-      <c r="C20" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="241" t="s">
+      <c r="C20" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="240" t="s">
         <v>2644</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="242" t="s">
+    <row r="21" spans="1:4" ht="12">
+      <c r="A21" s="245" t="s">
         <v>2720</v>
       </c>
-      <c r="B21" s="242" t="s">
+      <c r="B21" s="245" t="s">
         <v>2737</v>
       </c>
-      <c r="C21" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="241" t="s">
+      <c r="C21" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="240" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="242" t="s">
+    <row r="22" spans="1:4" ht="12">
+      <c r="A22" s="245" t="s">
         <v>2177</v>
       </c>
-      <c r="B22" s="242" t="s">
+      <c r="B22" s="245" t="s">
         <v>2738</v>
       </c>
-      <c r="C22" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D22" s="241" t="s">
+      <c r="C22" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D22" s="240" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="242" t="s">
+    <row r="23" spans="1:4" ht="12">
+      <c r="A23" s="245" t="s">
         <v>2721</v>
       </c>
-      <c r="B23" s="242" t="s">
+      <c r="B23" s="245" t="s">
         <v>2739</v>
       </c>
-      <c r="C23" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23" s="241" t="s">
+      <c r="C23" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" s="240" t="s">
         <v>2655</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="241" t="s">
+    <row r="24" spans="1:4" ht="12">
+      <c r="A24" s="240" t="s">
         <v>2656</v>
       </c>
-      <c r="B24" s="241" t="s">
+      <c r="B24" s="240" t="s">
         <v>2740</v>
       </c>
-      <c r="C24" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D24" s="241" t="s">
+      <c r="C24" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" s="240" t="s">
         <v>2660</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
-      <c r="A25" s="241" t="s">
+    <row r="25" spans="1:4" ht="12">
+      <c r="A25" s="240" t="s">
         <v>2710</v>
       </c>
-      <c r="B25" s="238" t="s">
+      <c r="B25" s="241" t="s">
         <v>2741</v>
       </c>
-      <c r="C25" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="241" t="s">
+      <c r="C25" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="240" t="s">
         <v>2660</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="241" t="s">
+    <row r="26" spans="1:4" ht="12">
+      <c r="A26" s="240" t="s">
         <v>2712</v>
       </c>
-      <c r="B26" s="238" t="s">
+      <c r="B26" s="241" t="s">
         <v>2742</v>
       </c>
-      <c r="C26" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D26" s="241" t="s">
+      <c r="C26" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" s="240" t="s">
         <v>2662</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="242" t="s">
+    <row r="27" spans="1:4" ht="12">
+      <c r="A27" s="245" t="s">
         <v>2663</v>
       </c>
-      <c r="B27" s="241" t="s">
+      <c r="B27" s="240" t="s">
         <v>2743</v>
       </c>
-      <c r="C27" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D27" s="241" t="s">
+      <c r="C27" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D27" s="240" t="s">
         <v>2666</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="242" t="s">
+    <row r="28" spans="1:4" ht="12">
+      <c r="A28" s="245" t="s">
         <v>2722</v>
       </c>
-      <c r="B28" s="242" t="s">
+      <c r="B28" s="245" t="s">
         <v>2744</v>
       </c>
-      <c r="C28" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D28" s="241" t="s">
+      <c r="C28" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="240" t="s">
         <v>2666</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="241" t="s">
+    <row r="29" spans="1:4" ht="12">
+      <c r="A29" s="240" t="s">
         <v>2718</v>
       </c>
-      <c r="B29" s="238" t="s">
+      <c r="B29" s="241" t="s">
         <v>2745</v>
       </c>
-      <c r="C29" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D29" s="241" t="s">
+      <c r="C29" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" s="240" t="s">
         <v>2667</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="241" t="s">
+    <row r="30" spans="1:4" ht="12">
+      <c r="A30" s="240" t="s">
         <v>2697</v>
       </c>
-      <c r="B30" s="241" t="s">
+      <c r="B30" s="240" t="s">
         <v>2746</v>
       </c>
-      <c r="C30" s="241" t="s">
-        <v>28</v>
-      </c>
-      <c r="D30" s="241" t="s">
+      <c r="C30" s="240" t="s">
+        <v>28</v>
+      </c>
+      <c r="D30" s="240" t="s">
         <v>2089</v>
       </c>
     </row>
@@ -17887,20 +17892,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17">
-      <c r="A1" s="233" t="s">
+      <c r="A1" s="236" t="s">
         <v>2346</v>
       </c>
-      <c r="B1" s="232"/>
-      <c r="C1" s="232"/>
-      <c r="D1" s="232"/>
+      <c r="B1" s="235"/>
+      <c r="C1" s="235"/>
+      <c r="D1" s="235"/>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="234" t="s">
+      <c r="A2" s="237" t="s">
         <v>2347</v>
       </c>
-      <c r="B2" s="232"/>
-      <c r="C2" s="232"/>
-      <c r="D2" s="232"/>
+      <c r="B2" s="235"/>
+      <c r="C2" s="235"/>
+      <c r="D2" s="235"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="181" t="s">
@@ -17917,12 +17922,12 @@
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="231" t="s">
+      <c r="A4" s="234" t="s">
         <v>2349</v>
       </c>
-      <c r="B4" s="232"/>
-      <c r="C4" s="232"/>
-      <c r="D4" s="232"/>
+      <c r="B4" s="235"/>
+      <c r="C4" s="235"/>
+      <c r="D4" s="235"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="182" t="s">
@@ -18149,12 +18154,12 @@
       </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="231" t="s">
+      <c r="A21" s="234" t="s">
         <v>2377</v>
       </c>
-      <c r="B21" s="232"/>
-      <c r="C21" s="232"/>
-      <c r="D21" s="232"/>
+      <c r="B21" s="235"/>
+      <c r="C21" s="235"/>
+      <c r="D21" s="235"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="186" t="s">
@@ -18199,12 +18204,12 @@
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="231" t="s">
+      <c r="A25" s="234" t="s">
         <v>2384</v>
       </c>
-      <c r="B25" s="232"/>
-      <c r="C25" s="232"/>
-      <c r="D25" s="232"/>
+      <c r="B25" s="235"/>
+      <c r="C25" s="235"/>
+      <c r="D25" s="235"/>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="186" t="s">
@@ -18249,12 +18254,12 @@
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="231" t="s">
+      <c r="A29" s="234" t="s">
         <v>2391</v>
       </c>
-      <c r="B29" s="232"/>
-      <c r="C29" s="232"/>
-      <c r="D29" s="232"/>
+      <c r="B29" s="235"/>
+      <c r="C29" s="235"/>
+      <c r="D29" s="235"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="186" t="s">
@@ -18299,12 +18304,12 @@
       </c>
     </row>
     <row r="33" spans="1:4">
-      <c r="A33" s="231" t="s">
+      <c r="A33" s="234" t="s">
         <v>2395</v>
       </c>
-      <c r="B33" s="232"/>
-      <c r="C33" s="232"/>
-      <c r="D33" s="232"/>
+      <c r="B33" s="235"/>
+      <c r="C33" s="235"/>
+      <c r="D33" s="235"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="186" t="s">
@@ -18363,12 +18368,12 @@
       </c>
     </row>
     <row r="38" spans="1:4">
-      <c r="A38" s="231" t="s">
+      <c r="A38" s="234" t="s">
         <v>2403</v>
       </c>
-      <c r="B38" s="232"/>
-      <c r="C38" s="232"/>
-      <c r="D38" s="232"/>
+      <c r="B38" s="235"/>
+      <c r="C38" s="235"/>
+      <c r="D38" s="235"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="190" t="s">
@@ -18413,12 +18418,12 @@
       </c>
     </row>
     <row r="42" spans="1:4">
-      <c r="A42" s="231" t="s">
+      <c r="A42" s="234" t="s">
         <v>2410</v>
       </c>
-      <c r="B42" s="232"/>
-      <c r="C42" s="232"/>
-      <c r="D42" s="232"/>
+      <c r="B42" s="235"/>
+      <c r="C42" s="235"/>
+      <c r="D42" s="235"/>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="190" t="s">
@@ -18463,12 +18468,12 @@
       </c>
     </row>
     <row r="46" spans="1:4">
-      <c r="A46" s="231" t="s">
+      <c r="A46" s="234" t="s">
         <v>2417</v>
       </c>
-      <c r="B46" s="232"/>
-      <c r="C46" s="232"/>
-      <c r="D46" s="232"/>
+      <c r="B46" s="235"/>
+      <c r="C46" s="235"/>
+      <c r="D46" s="235"/>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="190" t="s">
@@ -18513,12 +18518,12 @@
       </c>
     </row>
     <row r="50" spans="1:4">
-      <c r="A50" s="231" t="s">
+      <c r="A50" s="234" t="s">
         <v>2424</v>
       </c>
-      <c r="B50" s="232"/>
-      <c r="C50" s="232"/>
-      <c r="D50" s="232"/>
+      <c r="B50" s="235"/>
+      <c r="C50" s="235"/>
+      <c r="D50" s="235"/>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="190" t="s">
@@ -18563,12 +18568,12 @@
       </c>
     </row>
     <row r="54" spans="1:4">
-      <c r="A54" s="231" t="s">
+      <c r="A54" s="234" t="s">
         <v>2431</v>
       </c>
-      <c r="B54" s="232"/>
-      <c r="C54" s="232"/>
-      <c r="D54" s="232"/>
+      <c r="B54" s="235"/>
+      <c r="C54" s="235"/>
+      <c r="D54" s="235"/>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="190" t="s">
@@ -18613,12 +18618,12 @@
       </c>
     </row>
     <row r="58" spans="1:4">
-      <c r="A58" s="231" t="s">
+      <c r="A58" s="234" t="s">
         <v>2437</v>
       </c>
-      <c r="B58" s="232"/>
-      <c r="C58" s="232"/>
-      <c r="D58" s="232"/>
+      <c r="B58" s="235"/>
+      <c r="C58" s="235"/>
+      <c r="D58" s="235"/>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="190" t="s">
@@ -18663,12 +18668,12 @@
       </c>
     </row>
     <row r="62" spans="1:4">
-      <c r="A62" s="231" t="s">
+      <c r="A62" s="234" t="s">
         <v>2444</v>
       </c>
-      <c r="B62" s="232"/>
-      <c r="C62" s="232"/>
-      <c r="D62" s="232"/>
+      <c r="B62" s="235"/>
+      <c r="C62" s="235"/>
+      <c r="D62" s="235"/>
     </row>
     <row r="63" spans="1:4">
       <c r="A63" s="190" t="s">
@@ -18699,12 +18704,12 @@
       </c>
     </row>
     <row r="65" spans="1:4">
-      <c r="A65" s="231" t="s">
+      <c r="A65" s="234" t="s">
         <v>2449</v>
       </c>
-      <c r="B65" s="232"/>
-      <c r="C65" s="232"/>
-      <c r="D65" s="232"/>
+      <c r="B65" s="235"/>
+      <c r="C65" s="235"/>
+      <c r="D65" s="235"/>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="186" t="s">
@@ -18749,12 +18754,12 @@
       </c>
     </row>
     <row r="69" spans="1:4">
-      <c r="A69" s="231" t="s">
+      <c r="A69" s="234" t="s">
         <v>2455</v>
       </c>
-      <c r="B69" s="232"/>
-      <c r="C69" s="232"/>
-      <c r="D69" s="232"/>
+      <c r="B69" s="235"/>
+      <c r="C69" s="235"/>
+      <c r="D69" s="235"/>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="186" t="s">
@@ -18785,12 +18790,12 @@
       </c>
     </row>
     <row r="72" spans="1:4">
-      <c r="A72" s="231" t="s">
+      <c r="A72" s="234" t="s">
         <v>2460</v>
       </c>
-      <c r="B72" s="232"/>
-      <c r="C72" s="232"/>
-      <c r="D72" s="232"/>
+      <c r="B72" s="235"/>
+      <c r="C72" s="235"/>
+      <c r="D72" s="235"/>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="190" t="s">
@@ -18835,12 +18840,12 @@
       </c>
     </row>
     <row r="76" spans="1:4">
-      <c r="A76" s="231" t="s">
+      <c r="A76" s="234" t="s">
         <v>2467</v>
       </c>
-      <c r="B76" s="232"/>
-      <c r="C76" s="232"/>
-      <c r="D76" s="232"/>
+      <c r="B76" s="235"/>
+      <c r="C76" s="235"/>
+      <c r="D76" s="235"/>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="190" t="s">
@@ -18885,12 +18890,12 @@
       </c>
     </row>
     <row r="80" spans="1:4">
-      <c r="A80" s="231" t="s">
+      <c r="A80" s="234" t="s">
         <v>2474</v>
       </c>
-      <c r="B80" s="232"/>
-      <c r="C80" s="232"/>
-      <c r="D80" s="232"/>
+      <c r="B80" s="235"/>
+      <c r="C80" s="235"/>
+      <c r="D80" s="235"/>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="190" t="s">
@@ -18936,13 +18941,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A80:D80"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A62:D62"/>
-    <mergeCell ref="A65:D65"/>
-    <mergeCell ref="A69:D69"/>
-    <mergeCell ref="A72:D72"/>
-    <mergeCell ref="A76:D76"/>
     <mergeCell ref="A54:D54"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -18955,6 +18953,13 @@
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="A46:D46"/>
     <mergeCell ref="A50:D50"/>
+    <mergeCell ref="A80:D80"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A69:D69"/>
+    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="A76:D76"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>